<commit_message>
Update API configuration and InKindDonation component to use API_BASE_URL
</commit_message>
<xml_diff>
--- a/server/excel-logs/donations-2025-04.xlsx
+++ b/server/excel-logs/donations-2025-04.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -700,9 +700,38 @@
         <v>$30.00</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>MSC-0014</v>
+      </c>
+      <c r="B11" t="str">
+        <v>04/23/2025</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Taylor</v>
+      </c>
+      <c r="E11" t="str">
+        <v>ajgregojr@iu.edu</v>
+      </c>
+      <c r="F11" t="str">
+        <v>(317) 625-9575</v>
+      </c>
+      <c r="G11" t="str">
+        <v>7903 Pine Lake Road</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>$777.00</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>